<commit_message>
fix(seep04): the tutorial pair declares Time = s
If the time base is seconds, say so (owner's ruling — same as the SI
round's steady samples declaring yr). The builder sets time_unit on
both files, every label follows (k1 (m/s), Flux value (m/s), discharge
titles), the affected figures and the BC-editor shot regenerate, and
the page's paragraph explaining a blank Time field dies — it was prose
around a file that should simply have declared its unit.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_dam_infiltration.xlsx
+++ b/docs/tutorials/files/xslope_dam_infiltration.xlsx
@@ -2824,7 +2824,11 @@
       <c r="C9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="1"/>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="F9" s="1" t="s">
         <v>12</v>
       </c>

</xml_diff>